<commit_message>
Crawlability audit: final verification fixes
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/crawlability-bespirit-september-2026.xlsx
+++ b/public/crawlability-bespirit-september-2026.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -632,7 +632,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>karkur.bespirit.co.il: להסיר את הרשומה ב-DNS או להגדיר noindex.</t>
+          <t>להסיר ממפת האתר כתובות של דומיין אחר (landings.bespirit.co.il) או להגישן מהדומיין שלהן.</t>
         </is>
       </c>
     </row>
@@ -646,6 +646,21 @@
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>karkur.bespirit.co.il: להסיר את הרשומה ב-DNS או להגדיר noindex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>נמוכה</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>old.bespirit.co.il: עמוד ברירת מחדל של שרת. להסיר את הרשומה ב-DNS או להגדיר noindex.</t>
         </is>

</xml_diff>